<commit_message>
fix: complete data enlargement
</commit_message>
<xml_diff>
--- a/data/proteomics/ProMassRatio_across_compartment_NCB_yeast_IO.xlsx
+++ b/data/proteomics/ProMassRatio_across_compartment_NCB_yeast_IO.xlsx
@@ -1845,79 +1845,79 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0.01786106036338073</v>
+        <v>0.08356526920159377</v>
       </c>
       <c r="D17" t="n">
-        <v>0.01882880268990949</v>
+        <v>0.08667244113055705</v>
       </c>
       <c r="E17" t="n">
-        <v>0.01875826569990923</v>
+        <v>0.08947314930420019</v>
       </c>
       <c r="F17" t="n">
-        <v>0.01730604800221415</v>
+        <v>0.08923208938387753</v>
       </c>
       <c r="G17" t="n">
-        <v>0.01686389198958723</v>
+        <v>0.09092010254167404</v>
       </c>
       <c r="H17" t="n">
-        <v>0.01527260446865557</v>
+        <v>0.09404887879475653</v>
       </c>
       <c r="I17" t="n">
-        <v>0.02635421266347217</v>
+        <v>0.08401959534580429</v>
       </c>
       <c r="J17" t="n">
-        <v>0.02453846908255389</v>
+        <v>0.08285098511494514</v>
       </c>
       <c r="K17" t="n">
-        <v>0.02211656411103568</v>
+        <v>0.08995632560541691</v>
       </c>
       <c r="L17" t="n">
-        <v>0.01699424165730548</v>
+        <v>0.0916884698431453</v>
       </c>
       <c r="M17" t="n">
-        <v>0.01606459868445551</v>
+        <v>0.09424826591313738</v>
       </c>
       <c r="N17" t="n">
-        <v>0.02232668933898241</v>
+        <v>0.08631558859130906</v>
       </c>
       <c r="O17" t="n">
-        <v>0.02125102446944362</v>
+        <v>0.08574878259881775</v>
       </c>
       <c r="P17" t="n">
-        <v>0.01865311589028627</v>
+        <v>0.08796847735653357</v>
       </c>
       <c r="Q17" t="n">
-        <v>0.01443390366308459</v>
+        <v>0.09156846126679119</v>
       </c>
       <c r="R17" t="n">
-        <v>0.01155668496195075</v>
+        <v>0.08893794659086421</v>
       </c>
       <c r="S17" t="n">
-        <v>0.018137673046273</v>
+        <v>0.08932334463694416</v>
       </c>
       <c r="T17" t="n">
-        <v>0.0166828967506905</v>
+        <v>0.08987740928119697</v>
       </c>
       <c r="U17" t="n">
-        <v>0.01479784738807834</v>
+        <v>0.07103322894203359</v>
       </c>
       <c r="V17" t="n">
-        <v>0.007871793942612422</v>
+        <v>0.06138715468607484</v>
       </c>
       <c r="W17" t="n">
-        <v>0.007605670513354018</v>
+        <v>0.05462878621527467</v>
       </c>
       <c r="X17" t="n">
-        <v>0.00790426052973792</v>
+        <v>0.05264332333677837</v>
       </c>
       <c r="Y17" t="n">
-        <v>0.01854044664682626</v>
+        <v>0.103957577999024</v>
       </c>
       <c r="Z17" t="n">
-        <v>0.01890625293588711</v>
+        <v>0.1066882173928116</v>
       </c>
       <c r="AA17" t="n">
-        <v>0.0150176595212246</v>
+        <v>0.08146079775277605</v>
       </c>
     </row>
     <row r="18">

</xml_diff>